<commit_message>
debug: 在 _resume_pending_records 中添加更多调试日志
添加调试日志追踪 _request_evaluation 的调用过程，
帮助确定消息发送流程中的问题所在。

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/records/初始试模清单.xlsx
+++ b/data/records/初始试模清单.xlsx
@@ -480,31 +480,31 @@
     </row>
     <row r="2">
       <c r="A2" t="n">
-        <v>142</v>
+        <v>138</v>
       </c>
       <c r="B2" t="n">
-        <v>700</v>
+        <v>860</v>
       </c>
       <c r="C2" t="n">
-        <v>380</v>
+        <v>460</v>
       </c>
       <c r="D2" t="n">
-        <v>1</v>
+        <v>0.5</v>
       </c>
       <c r="E2" t="n">
+        <v>20</v>
+      </c>
+      <c r="F2" t="n">
         <v>35</v>
       </c>
-      <c r="F2" t="n">
-        <v>40</v>
-      </c>
       <c r="G2" t="n">
-        <v>10</v>
+        <v>25</v>
       </c>
       <c r="H2" t="n">
         <v>20</v>
       </c>
       <c r="I2" t="n">
-        <v>35</v>
+        <v>10</v>
       </c>
       <c r="J2" t="n">
         <v>16</v>
@@ -520,31 +520,31 @@
     </row>
     <row r="3">
       <c r="A3" t="n">
-        <v>138</v>
+        <v>140</v>
       </c>
       <c r="B3" t="n">
-        <v>1000</v>
+        <v>1060</v>
       </c>
       <c r="C3" t="n">
-        <v>520</v>
+        <v>360</v>
       </c>
       <c r="D3" t="n">
-        <v>1.5</v>
+        <v>2</v>
       </c>
       <c r="E3" t="n">
-        <v>10</v>
+        <v>35</v>
       </c>
       <c r="F3" t="n">
-        <v>20</v>
+        <v>10</v>
       </c>
       <c r="G3" t="n">
-        <v>25</v>
+        <v>15</v>
       </c>
       <c r="H3" t="n">
-        <v>25</v>
+        <v>30</v>
       </c>
       <c r="I3" t="n">
-        <v>5</v>
+        <v>35</v>
       </c>
       <c r="J3" t="n">
         <v>16</v>
@@ -560,31 +560,31 @@
     </row>
     <row r="4">
       <c r="A4" t="n">
-        <v>137</v>
+        <v>143</v>
       </c>
       <c r="B4" t="n">
-        <v>840</v>
+        <v>760</v>
       </c>
       <c r="C4" t="n">
-        <v>340</v>
+        <v>600</v>
       </c>
       <c r="D4" t="n">
-        <v>0.5</v>
+        <v>0</v>
       </c>
       <c r="E4" t="n">
-        <v>15</v>
+        <v>25</v>
       </c>
       <c r="F4" t="n">
-        <v>5</v>
+        <v>20</v>
       </c>
       <c r="G4" t="n">
-        <v>20</v>
+        <v>40</v>
       </c>
       <c r="H4" t="n">
-        <v>35</v>
+        <v>40</v>
       </c>
       <c r="I4" t="n">
-        <v>15</v>
+        <v>30</v>
       </c>
       <c r="J4" t="n">
         <v>16</v>
@@ -600,31 +600,31 @@
     </row>
     <row r="5">
       <c r="A5" t="n">
-        <v>141</v>
+        <v>137</v>
       </c>
       <c r="B5" t="n">
-        <v>1140</v>
+        <v>1080</v>
       </c>
       <c r="C5" t="n">
-        <v>480</v>
+        <v>320</v>
       </c>
       <c r="D5" t="n">
-        <v>2</v>
+        <v>1.5</v>
       </c>
       <c r="E5" t="n">
-        <v>25</v>
+        <v>10</v>
       </c>
       <c r="F5" t="n">
         <v>25</v>
       </c>
       <c r="G5" t="n">
-        <v>35</v>
+        <v>10</v>
       </c>
       <c r="H5" t="n">
-        <v>15</v>
+        <v>10</v>
       </c>
       <c r="I5" t="n">
-        <v>25</v>
+        <v>20</v>
       </c>
       <c r="J5" t="n">
         <v>16</v>
@@ -640,31 +640,31 @@
     </row>
     <row r="6">
       <c r="A6" t="n">
-        <v>140</v>
+        <v>136</v>
       </c>
       <c r="B6" t="n">
-        <v>880</v>
+        <v>760</v>
       </c>
       <c r="C6" t="n">
-        <v>580</v>
+        <v>420</v>
       </c>
       <c r="D6" t="n">
-        <v>1.5</v>
+        <v>1</v>
       </c>
       <c r="E6" t="n">
-        <v>30</v>
+        <v>10</v>
       </c>
       <c r="F6" t="n">
         <v>35</v>
       </c>
       <c r="G6" t="n">
-        <v>15</v>
+        <v>35</v>
       </c>
       <c r="H6" t="n">
-        <v>35</v>
+        <v>30</v>
       </c>
       <c r="I6" t="n">
-        <v>20</v>
+        <v>25</v>
       </c>
       <c r="J6" t="n">
         <v>16</v>
@@ -680,31 +680,31 @@
     </row>
     <row r="7">
       <c r="A7" t="n">
-        <v>136</v>
+        <v>142</v>
       </c>
       <c r="B7" t="n">
         <v>1200</v>
       </c>
       <c r="C7" t="n">
-        <v>400</v>
+        <v>500</v>
       </c>
       <c r="D7" t="n">
-        <v>0</v>
+        <v>0.5</v>
       </c>
       <c r="E7" t="n">
-        <v>20</v>
+        <v>25</v>
       </c>
       <c r="F7" t="n">
-        <v>15</v>
+        <v>10</v>
       </c>
       <c r="G7" t="n">
-        <v>30</v>
+        <v>10</v>
       </c>
       <c r="H7" t="n">
-        <v>5</v>
+        <v>10</v>
       </c>
       <c r="I7" t="n">
-        <v>30</v>
+        <v>20</v>
       </c>
       <c r="J7" t="n">
         <v>16</v>
@@ -720,31 +720,31 @@
     </row>
     <row r="8">
       <c r="A8" t="n">
-        <v>139</v>
+        <v>141</v>
       </c>
       <c r="B8" t="n">
-        <v>760</v>
+        <v>900</v>
       </c>
       <c r="C8" t="n">
-        <v>440</v>
+        <v>280</v>
       </c>
       <c r="D8" t="n">
-        <v>1</v>
+        <v>1.5</v>
       </c>
       <c r="E8" t="n">
+        <v>35</v>
+      </c>
+      <c r="F8" t="n">
         <v>15</v>
       </c>
-      <c r="F8" t="n">
-        <v>10</v>
-      </c>
       <c r="G8" t="n">
-        <v>5</v>
+        <v>30</v>
       </c>
       <c r="H8" t="n">
-        <v>15</v>
+        <v>20</v>
       </c>
       <c r="I8" t="n">
-        <v>35</v>
+        <v>10</v>
       </c>
       <c r="J8" t="n">
         <v>16</v>
@@ -760,31 +760,31 @@
     </row>
     <row r="9">
       <c r="A9" t="n">
-        <v>143</v>
+        <v>139</v>
       </c>
       <c r="B9" t="n">
-        <v>1080</v>
+        <v>960</v>
       </c>
       <c r="C9" t="n">
-        <v>260</v>
+        <v>540</v>
       </c>
       <c r="D9" t="n">
-        <v>0.5</v>
+        <v>1</v>
       </c>
       <c r="E9" t="n">
-        <v>40</v>
+        <v>20</v>
       </c>
       <c r="F9" t="n">
         <v>30</v>
       </c>
       <c r="G9" t="n">
+        <v>20</v>
+      </c>
+      <c r="H9" t="n">
         <v>25</v>
       </c>
-      <c r="H9" t="n">
-        <v>30</v>
-      </c>
       <c r="I9" t="n">
-        <v>15</v>
+        <v>35</v>
       </c>
       <c r="J9" t="n">
         <v>16</v>
@@ -800,31 +800,31 @@
     </row>
     <row r="10">
       <c r="A10" t="n">
-        <v>142</v>
+        <v>139</v>
       </c>
       <c r="B10" t="n">
-        <v>860</v>
+        <v>820</v>
       </c>
       <c r="C10" t="n">
-        <v>440</v>
+        <v>260</v>
       </c>
       <c r="D10" t="n">
-        <v>0</v>
+        <v>0.5</v>
       </c>
       <c r="E10" t="n">
-        <v>5</v>
+        <v>40</v>
       </c>
       <c r="F10" t="n">
         <v>25</v>
       </c>
       <c r="G10" t="n">
-        <v>15</v>
+        <v>30</v>
       </c>
       <c r="H10" t="n">
-        <v>40</v>
+        <v>35</v>
       </c>
       <c r="I10" t="n">
-        <v>20</v>
+        <v>25</v>
       </c>
       <c r="J10" t="n">
         <v>16</v>
@@ -840,31 +840,31 @@
     </row>
     <row r="11">
       <c r="A11" t="n">
-        <v>139</v>
+        <v>141</v>
       </c>
       <c r="B11" t="n">
-        <v>1100</v>
+        <v>1120</v>
       </c>
       <c r="C11" t="n">
-        <v>280</v>
+        <v>540</v>
       </c>
       <c r="D11" t="n">
-        <v>1.5</v>
+        <v>1</v>
       </c>
       <c r="E11" t="n">
-        <v>30</v>
+        <v>20</v>
       </c>
       <c r="F11" t="n">
-        <v>10</v>
+        <v>20</v>
       </c>
       <c r="G11" t="n">
-        <v>35</v>
+        <v>5</v>
       </c>
       <c r="H11" t="n">
-        <v>10</v>
+        <v>5</v>
       </c>
       <c r="I11" t="n">
-        <v>30</v>
+        <v>15</v>
       </c>
       <c r="J11" t="n">
         <v>16</v>

</xml_diff>

<commit_message>
fix: 修复 BayesianOptimizer 导入错误
__init__.py 尝试导入不存在的 BayesianOptimizer 类，
实际定义的类是 StandardBOOptimizer。

修改文件：
- src/injection_molding/core/bayesian/__init__.py
- src/injection_molding/core/__init__.py

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/records/初始试模清单.xlsx
+++ b/data/records/初始试模清单.xlsx
@@ -480,13 +480,13 @@
     </row>
     <row r="2">
       <c r="A2" t="n">
-        <v>142</v>
+        <v>143</v>
       </c>
       <c r="B2" t="n">
-        <v>1120</v>
+        <v>960</v>
       </c>
       <c r="C2" t="n">
-        <v>340</v>
+        <v>540</v>
       </c>
       <c r="D2" t="n">
         <v>0</v>
@@ -495,13 +495,13 @@
         <v>10</v>
       </c>
       <c r="F2" t="n">
-        <v>10</v>
+        <v>40</v>
       </c>
       <c r="G2" t="n">
+        <v>35</v>
+      </c>
+      <c r="H2" t="n">
         <v>25</v>
-      </c>
-      <c r="H2" t="n">
-        <v>30</v>
       </c>
       <c r="I2" t="n">
         <v>35</v>
@@ -523,28 +523,28 @@
         <v>138</v>
       </c>
       <c r="B3" t="n">
-        <v>760</v>
+        <v>920</v>
       </c>
       <c r="C3" t="n">
-        <v>560</v>
+        <v>420</v>
       </c>
       <c r="D3" t="n">
-        <v>1.5</v>
+        <v>2</v>
       </c>
       <c r="E3" t="n">
-        <v>25</v>
+        <v>30</v>
       </c>
       <c r="F3" t="n">
-        <v>30</v>
+        <v>10</v>
       </c>
       <c r="G3" t="n">
-        <v>20</v>
+        <v>10</v>
       </c>
       <c r="H3" t="n">
+        <v>10</v>
+      </c>
+      <c r="I3" t="n">
         <v>5</v>
-      </c>
-      <c r="I3" t="n">
-        <v>20</v>
       </c>
       <c r="J3" t="n">
         <v>16</v>
@@ -560,31 +560,31 @@
     </row>
     <row r="4">
       <c r="A4" t="n">
-        <v>138</v>
+        <v>136</v>
       </c>
       <c r="B4" t="n">
-        <v>960</v>
+        <v>1120</v>
       </c>
       <c r="C4" t="n">
-        <v>280</v>
+        <v>480</v>
       </c>
       <c r="D4" t="n">
-        <v>1</v>
+        <v>0.5</v>
       </c>
       <c r="E4" t="n">
-        <v>35</v>
+        <v>40</v>
       </c>
       <c r="F4" t="n">
-        <v>40</v>
+        <v>20</v>
       </c>
       <c r="G4" t="n">
-        <v>35</v>
+        <v>25</v>
       </c>
       <c r="H4" t="n">
         <v>20</v>
       </c>
       <c r="I4" t="n">
-        <v>10</v>
+        <v>20</v>
       </c>
       <c r="J4" t="n">
         <v>16</v>
@@ -600,13 +600,13 @@
     </row>
     <row r="5">
       <c r="A5" t="n">
-        <v>140</v>
+        <v>141</v>
       </c>
       <c r="B5" t="n">
-        <v>840</v>
+        <v>780</v>
       </c>
       <c r="C5" t="n">
-        <v>500</v>
+        <v>260</v>
       </c>
       <c r="D5" t="n">
         <v>1.5</v>
@@ -615,16 +615,16 @@
         <v>15</v>
       </c>
       <c r="F5" t="n">
-        <v>20</v>
+        <v>25</v>
       </c>
       <c r="G5" t="n">
         <v>15</v>
       </c>
       <c r="H5" t="n">
+        <v>35</v>
+      </c>
+      <c r="I5" t="n">
         <v>30</v>
-      </c>
-      <c r="I5" t="n">
-        <v>25</v>
       </c>
       <c r="J5" t="n">
         <v>16</v>
@@ -640,13 +640,13 @@
     </row>
     <row r="6">
       <c r="A6" t="n">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="B6" t="n">
-        <v>1040</v>
+        <v>1160</v>
       </c>
       <c r="C6" t="n">
-        <v>520</v>
+        <v>360</v>
       </c>
       <c r="D6" t="n">
         <v>1</v>
@@ -655,16 +655,16 @@
         <v>20</v>
       </c>
       <c r="F6" t="n">
-        <v>10</v>
+        <v>35</v>
       </c>
       <c r="G6" t="n">
-        <v>40</v>
+        <v>30</v>
       </c>
       <c r="H6" t="n">
         <v>15</v>
       </c>
       <c r="I6" t="n">
-        <v>10</v>
+        <v>15</v>
       </c>
       <c r="J6" t="n">
         <v>16</v>
@@ -680,28 +680,28 @@
     </row>
     <row r="7">
       <c r="A7" t="n">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="B7" t="n">
-        <v>900</v>
+        <v>760</v>
       </c>
       <c r="C7" t="n">
-        <v>380</v>
+        <v>600</v>
       </c>
       <c r="D7" t="n">
-        <v>0.5</v>
+        <v>1</v>
       </c>
       <c r="E7" t="n">
         <v>30</v>
       </c>
       <c r="F7" t="n">
-        <v>25</v>
+        <v>5</v>
       </c>
       <c r="G7" t="n">
-        <v>5</v>
+        <v>20</v>
       </c>
       <c r="H7" t="n">
-        <v>25</v>
+        <v>35</v>
       </c>
       <c r="I7" t="n">
         <v>25</v>
@@ -723,25 +723,25 @@
         <v>139</v>
       </c>
       <c r="B8" t="n">
-        <v>1200</v>
+        <v>1040</v>
       </c>
       <c r="C8" t="n">
-        <v>440</v>
+        <v>320</v>
       </c>
       <c r="D8" t="n">
-        <v>2</v>
+        <v>1.5</v>
       </c>
       <c r="E8" t="n">
+        <v>25</v>
+      </c>
+      <c r="F8" t="n">
+        <v>20</v>
+      </c>
+      <c r="G8" t="n">
+        <v>40</v>
+      </c>
+      <c r="H8" t="n">
         <v>30</v>
-      </c>
-      <c r="F8" t="n">
-        <v>30</v>
-      </c>
-      <c r="G8" t="n">
-        <v>25</v>
-      </c>
-      <c r="H8" t="n">
-        <v>35</v>
       </c>
       <c r="I8" t="n">
         <v>35</v>
@@ -763,25 +763,25 @@
         <v>142</v>
       </c>
       <c r="B9" t="n">
-        <v>800</v>
+        <v>840</v>
       </c>
       <c r="C9" t="n">
-        <v>320</v>
+        <v>440</v>
       </c>
       <c r="D9" t="n">
         <v>0.5</v>
       </c>
       <c r="E9" t="n">
+        <v>10</v>
+      </c>
+      <c r="F9" t="n">
+        <v>25</v>
+      </c>
+      <c r="G9" t="n">
+        <v>10</v>
+      </c>
+      <c r="H9" t="n">
         <v>5</v>
-      </c>
-      <c r="F9" t="n">
-        <v>20</v>
-      </c>
-      <c r="G9" t="n">
-        <v>15</v>
-      </c>
-      <c r="H9" t="n">
-        <v>10</v>
       </c>
       <c r="I9" t="n">
         <v>15</v>
@@ -803,28 +803,28 @@
         <v>141</v>
       </c>
       <c r="B10" t="n">
-        <v>1000</v>
+        <v>1080</v>
       </c>
       <c r="C10" t="n">
-        <v>440</v>
+        <v>320</v>
       </c>
       <c r="D10" t="n">
-        <v>0.5</v>
+        <v>1</v>
       </c>
       <c r="E10" t="n">
-        <v>25</v>
+        <v>30</v>
       </c>
       <c r="F10" t="n">
-        <v>20</v>
+        <v>30</v>
       </c>
       <c r="G10" t="n">
-        <v>35</v>
+        <v>30</v>
       </c>
       <c r="H10" t="n">
-        <v>20</v>
+        <v>15</v>
       </c>
       <c r="I10" t="n">
-        <v>5</v>
+        <v>15</v>
       </c>
       <c r="J10" t="n">
         <v>16</v>
@@ -843,28 +843,28 @@
         <v>139</v>
       </c>
       <c r="B11" t="n">
-        <v>860</v>
+        <v>800</v>
       </c>
       <c r="C11" t="n">
-        <v>320</v>
+        <v>460</v>
       </c>
       <c r="D11" t="n">
         <v>1</v>
       </c>
       <c r="E11" t="n">
-        <v>15</v>
+        <v>5</v>
       </c>
       <c r="F11" t="n">
+        <v>20</v>
+      </c>
+      <c r="G11" t="n">
+        <v>20</v>
+      </c>
+      <c r="H11" t="n">
         <v>40</v>
       </c>
-      <c r="G11" t="n">
-        <v>5</v>
-      </c>
-      <c r="H11" t="n">
+      <c r="I11" t="n">
         <v>25</v>
-      </c>
-      <c r="I11" t="n">
-        <v>30</v>
       </c>
       <c r="J11" t="n">
         <v>16</v>

</xml_diff>